<commit_message>
PicoDebugBoard B0 revision after correcting minor bugs in the design
</commit_message>
<xml_diff>
--- a/SensWear-V1R2-Debug/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R2-Debug.xlsx
+++ b/SensWear-V1R2-Debug/Output/Manufacturing/Assembly/Bill of Materials/Bill of Materials-SensWear-V1R2-Debug.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\WORK\Projects\SensWear\hardware-v1\SensWear-V1R2-Debug\Output\Manufacturing\Assembly\Bill of Materials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46CBEDD3-465B-40B0-B643-85F6CACE36E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1DD4CB7A-944D-4926-8C4F-85DB7E65C3F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3790" yWindow="3660" windowWidth="28800" windowHeight="17170" xr2:uid="{8B973B5F-F8C3-4C86-81CB-9745F1413E71}"/>
+    <workbookView xWindow="5700" yWindow="5700" windowWidth="28800" windowHeight="17170" xr2:uid="{1BF58602-27FE-45E4-983A-78381B6B1334}"/>
   </bookViews>
   <sheets>
     <sheet name="Bill of Materials-SensWear-V1R2" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="171">
   <si>
     <t>Manufacturer</t>
   </si>
@@ -212,319 +212,319 @@
     <t>490-1006-1-ND</t>
   </si>
   <si>
+    <t>DFE201612E-2R2M=P2</t>
+  </si>
+  <si>
+    <t>L50</t>
+  </si>
+  <si>
+    <t>2.2 uH</t>
+  </si>
+  <si>
+    <t>Inductor Power Shielded Wirewound 2.2uH 20% 1MHz Metal 1.8A 0.116Ohm DCR 0806 T/R</t>
+  </si>
+  <si>
+    <t>FP-DFE201612C-MFG</t>
+  </si>
+  <si>
+    <t>81-DFE201612E-2R2MP2</t>
+  </si>
+  <si>
+    <t>JAE Electronics</t>
+  </si>
+  <si>
+    <t>DX07S024JJ3R1300</t>
+  </si>
+  <si>
+    <t>USB50</t>
+  </si>
+  <si>
+    <t>Cut Tape - Usb Type C Receptacle Mid Mnt Dual R</t>
+  </si>
+  <si>
+    <t>JAE-DX07S024JJ3R1300-MFG</t>
+  </si>
+  <si>
+    <t>656-DX07S024JJ3R1300</t>
+  </si>
+  <si>
+    <t>Panasonic</t>
+  </si>
+  <si>
+    <t>ERJ2RKF2202X</t>
+  </si>
+  <si>
+    <t>R54</t>
+  </si>
+  <si>
+    <t>22kΩ</t>
+  </si>
+  <si>
+    <t>Res Thick Film 0402 22K Ohm 1% 0.1W(1/10W) ±100ppm/C Pad SMD Automotive T/R</t>
+  </si>
+  <si>
+    <t>RESC1005X04N</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF27R0X</t>
+  </si>
+  <si>
+    <t>R56, R58</t>
+  </si>
+  <si>
+    <t>27Ω</t>
+  </si>
+  <si>
+    <t>Res Thick Film 0402 27 Ohm 1% 0.1W ±100ppm/°C Molded SMD Punched Carrier T/R</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF33R0X</t>
+  </si>
+  <si>
+    <t>R57</t>
+  </si>
+  <si>
+    <t>33R</t>
+  </si>
+  <si>
+    <t>RES SMD 33 OHM 1% 1/10W 0402</t>
+  </si>
+  <si>
+    <t>667-ERJ-2RKF33R0X</t>
+  </si>
+  <si>
+    <t>Panasonic Electronic Components</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF1000X</t>
+  </si>
+  <si>
+    <t>R64, R65, R66, R67</t>
+  </si>
+  <si>
+    <t>100 R</t>
+  </si>
+  <si>
+    <t>RES SMD 100 OHM 1% 1/10W 0402</t>
+  </si>
+  <si>
+    <t>P100LDKR-ND</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF1001X</t>
+  </si>
+  <si>
+    <t>R59, R62, R63, R74, R75, R76, R77, R78, R79</t>
+  </si>
+  <si>
+    <t>1 k</t>
+  </si>
+  <si>
+    <t>RES SMD 1K OHM 1% 1/10W 0402</t>
+  </si>
+  <si>
+    <t>P1.00KLDKR-ND</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF2673X</t>
+  </si>
+  <si>
+    <t>R55</t>
+  </si>
+  <si>
+    <t>267kΩ</t>
+  </si>
+  <si>
+    <t>Res Thick Film 0402 267K Ohm 1% 1/10W ±100ppm/°C Molded SMD Punched Carrier T/R</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF5101X</t>
+  </si>
+  <si>
+    <t>R60, R61</t>
+  </si>
+  <si>
+    <t>5.1 k</t>
+  </si>
+  <si>
+    <t>RES SMD 5.1K OHM 1% 1/10W 0402</t>
+  </si>
+  <si>
+    <t>667-ERJ-2RKF5101X</t>
+  </si>
+  <si>
+    <t>ERJ-2RKF6200X</t>
+  </si>
+  <si>
+    <t>R68, R69, R70, R71, R72, R73</t>
+  </si>
+  <si>
+    <t>620 R</t>
+  </si>
+  <si>
+    <t>RES SMD 620 OHM 1% 1/10W 0402</t>
+  </si>
+  <si>
+    <t>P620LCT-ND</t>
+  </si>
+  <si>
+    <t>Fairchild Semiconductor</t>
+  </si>
+  <si>
+    <t>FPF1320UCX</t>
+  </si>
+  <si>
+    <t>U50</t>
+  </si>
+  <si>
+    <t>IC ADVANCED POWER SWITCH 6WLCSP</t>
+  </si>
+  <si>
+    <t>BGA6C50P2X3_96X146X62</t>
+  </si>
+  <si>
+    <t>FPF1320UCXDKR-ND</t>
+  </si>
+  <si>
+    <t>Murata Electronics North America</t>
+  </si>
+  <si>
+    <t>GRM155R61A104KA01D</t>
+  </si>
+  <si>
+    <t>C52, C53, C54, C55, C56, C57, C58, C59, C60, C61, C62, C63, C71, C72</t>
+  </si>
+  <si>
+    <t>0.1 uF</t>
+  </si>
+  <si>
+    <t>CAP CER 0.1UF 10V X5R 0402</t>
+  </si>
+  <si>
+    <t>CAPC1005X05N</t>
+  </si>
+  <si>
+    <t>490-1318-6-ND</t>
+  </si>
+  <si>
+    <t>GRM155R61A475MEAAD</t>
+  </si>
+  <si>
+    <t>C51</t>
+  </si>
+  <si>
+    <t>4.7uF</t>
+  </si>
+  <si>
+    <t>Multilayer Ceramic Capacitor, 4.7 uF, 10 V, ± 20%, X5R, 0402 [1005 Metric]</t>
+  </si>
+  <si>
+    <t>81-GRM155R61A475MEAD</t>
+  </si>
+  <si>
+    <t>GRM188R61A475KE15D</t>
+  </si>
+  <si>
+    <t>C50, C64, C65, C66, C67, C68</t>
+  </si>
+  <si>
+    <t>4.7 uF</t>
+  </si>
+  <si>
+    <t>CAP CER 4.7UF 10V X5R 0603</t>
+  </si>
+  <si>
+    <t>CAPC1610X05N</t>
+  </si>
+  <si>
+    <t>490-10477-6-ND</t>
+  </si>
+  <si>
+    <t>GRM1555C1E150JA01D</t>
+  </si>
+  <si>
+    <t>C69, C70</t>
+  </si>
+  <si>
+    <t>15pF</t>
+  </si>
+  <si>
+    <t>CAP CER 15 pF 25V C0G 0402</t>
+  </si>
+  <si>
+    <t>Vishay Lite-On</t>
+  </si>
+  <si>
+    <t>LTST-C155KGJRKT</t>
+  </si>
+  <si>
+    <t>D51, D52, D53</t>
+  </si>
+  <si>
+    <t>LED GREEN/RED CLEAR CHIP SMD</t>
+  </si>
+  <si>
+    <t>160-1409-1-ND</t>
+  </si>
+  <si>
+    <t>ON Semiconductor</t>
+  </si>
+  <si>
+    <t>MBR140SFT1G</t>
+  </si>
+  <si>
+    <t>D50</t>
+  </si>
+  <si>
+    <t>DIODE SCHOTTKY 40V 1A SOD123L</t>
+  </si>
+  <si>
+    <t>SODFL360X110-2N</t>
+  </si>
+  <si>
+    <t>MBR140SFT1GOSDKR-ND</t>
+  </si>
+  <si>
+    <t>onsemi</t>
+  </si>
+  <si>
+    <t>NTLJD4116NT1G</t>
+  </si>
+  <si>
+    <t>T50, T51, T52</t>
+  </si>
+  <si>
+    <t>NTLJD4116NT1G Dual N-channel Mosfet Transistor, 2.5 A, 30 V, 6-PIN Wdfn</t>
+  </si>
+  <si>
+    <t>FP-DQK0006B-MFG</t>
+  </si>
+  <si>
+    <t>Arrow Electronics</t>
+  </si>
+  <si>
+    <t>NXP Semiconductors</t>
+  </si>
+  <si>
+    <t>PRTR5V0U2F,115</t>
+  </si>
+  <si>
+    <t>U52</t>
+  </si>
+  <si>
+    <t>PRTR5V0U2F</t>
+  </si>
+  <si>
+    <t>TVS DIODE 5.5VWM SOT886</t>
+  </si>
+  <si>
+    <t>SON50P100X50-6N</t>
+  </si>
+  <si>
+    <t>568-4677-6-ND</t>
+  </si>
+  <si>
     <t>Texas Instruments</t>
-  </si>
-  <si>
-    <t>CSD87502Q2</t>
-  </si>
-  <si>
-    <t>T50, T51, T52</t>
-  </si>
-  <si>
-    <t>Transistor MOSFET Array Dual N-CH 30V 5A 6-Pin WSON T/R</t>
-  </si>
-  <si>
-    <t>FP-DQK0006B-MFG</t>
-  </si>
-  <si>
-    <t>296-48123-1-ND</t>
-  </si>
-  <si>
-    <t>DFE201612E-2R2M=P2</t>
-  </si>
-  <si>
-    <t>L50</t>
-  </si>
-  <si>
-    <t>2.2 uH</t>
-  </si>
-  <si>
-    <t>Inductor Power Shielded Wirewound 2.2uH 20% 1MHz Metal 1.8A 0.116Ohm DCR 0806 T/R</t>
-  </si>
-  <si>
-    <t>FP-DFE201612C-MFG</t>
-  </si>
-  <si>
-    <t>81-DFE201612E-2R2MP2</t>
-  </si>
-  <si>
-    <t>JAE Electronics</t>
-  </si>
-  <si>
-    <t>DX07S024JJ3R1300</t>
-  </si>
-  <si>
-    <t>USB50</t>
-  </si>
-  <si>
-    <t>Cut Tape - Usb Type C Receptacle Mid Mnt Dual R</t>
-  </si>
-  <si>
-    <t>JAE-DX07S024JJ3R1300-MFG</t>
-  </si>
-  <si>
-    <t>656-DX07S024JJ3R1300</t>
-  </si>
-  <si>
-    <t>Panasonic</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF27R0X</t>
-  </si>
-  <si>
-    <t>R56, R58</t>
-  </si>
-  <si>
-    <t>27Ω</t>
-  </si>
-  <si>
-    <t>Res Thick Film 0402 27 Ohm 1% 0.1W ±100ppm/°C Molded SMD Punched Carrier T/R</t>
-  </si>
-  <si>
-    <t>RESC1005X04N</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF33R0X</t>
-  </si>
-  <si>
-    <t>R57</t>
-  </si>
-  <si>
-    <t>33R</t>
-  </si>
-  <si>
-    <t>RES SMD 33 OHM 1% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>667-ERJ-2RKF33R0X</t>
-  </si>
-  <si>
-    <t>Panasonic Electronic Components</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF1000X</t>
-  </si>
-  <si>
-    <t>R64, R65, R66, R67</t>
-  </si>
-  <si>
-    <t>100 R</t>
-  </si>
-  <si>
-    <t>RES SMD 100 OHM 1% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>P100LDKR-ND</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF1001X</t>
-  </si>
-  <si>
-    <t>R59, R62, R63, R74, R75, R76, R77, R78, R79</t>
-  </si>
-  <si>
-    <t>1 k</t>
-  </si>
-  <si>
-    <t>RES SMD 1K OHM 1% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>P1.00KLDKR-ND</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF1004X</t>
-  </si>
-  <si>
-    <t>R54</t>
-  </si>
-  <si>
-    <t>1 M</t>
-  </si>
-  <si>
-    <t>RES SMD 1M OHM 1% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>P1.00MLDKR-ND</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF2673X</t>
-  </si>
-  <si>
-    <t>R55</t>
-  </si>
-  <si>
-    <t>267kΩ</t>
-  </si>
-  <si>
-    <t>Res Thick Film 0402 267K Ohm 1% 1/10W ±100ppm/°C Molded SMD Punched Carrier T/R</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF5101X</t>
-  </si>
-  <si>
-    <t>R60, R61</t>
-  </si>
-  <si>
-    <t>5.1 k</t>
-  </si>
-  <si>
-    <t>RES SMD 5.1K OHM 1% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>667-ERJ-2RKF5101X</t>
-  </si>
-  <si>
-    <t>ERJ-2RKF6200X</t>
-  </si>
-  <si>
-    <t>R68, R69, R70, R71, R72, R73</t>
-  </si>
-  <si>
-    <t>620 R</t>
-  </si>
-  <si>
-    <t>RES SMD 620 OHM 1% 1/10W 0402</t>
-  </si>
-  <si>
-    <t>P620LCT-ND</t>
-  </si>
-  <si>
-    <t>Fairchild Semiconductor</t>
-  </si>
-  <si>
-    <t>FPF1320UCX</t>
-  </si>
-  <si>
-    <t>U50</t>
-  </si>
-  <si>
-    <t>IC ADVANCED POWER SWITCH 6WLCSP</t>
-  </si>
-  <si>
-    <t>BGA6C50P2X3_96X146X62</t>
-  </si>
-  <si>
-    <t>FPF1320UCXDKR-ND</t>
-  </si>
-  <si>
-    <t>Murata Electronics North America</t>
-  </si>
-  <si>
-    <t>GRM155R61A104KA01D</t>
-  </si>
-  <si>
-    <t>C52, C53, C54, C55, C56, C57, C58, C59, C60, C61, C62, C63, C71, C72</t>
-  </si>
-  <si>
-    <t>0.1 uF</t>
-  </si>
-  <si>
-    <t>CAP CER 0.1UF 10V X5R 0402</t>
-  </si>
-  <si>
-    <t>CAPC1005X05N</t>
-  </si>
-  <si>
-    <t>490-1318-6-ND</t>
-  </si>
-  <si>
-    <t>GRM155R61A475MEAAD</t>
-  </si>
-  <si>
-    <t>C51</t>
-  </si>
-  <si>
-    <t>4.7uF</t>
-  </si>
-  <si>
-    <t>Multilayer Ceramic Capacitor, 4.7 uF, 10 V, ± 20%, X5R, 0402 [1005 Metric]</t>
-  </si>
-  <si>
-    <t>81-GRM155R61A475MEAD</t>
-  </si>
-  <si>
-    <t>GRM188R61A475KE15D</t>
-  </si>
-  <si>
-    <t>C50, C64, C65, C66, C67, C68</t>
-  </si>
-  <si>
-    <t>4.7 uF</t>
-  </si>
-  <si>
-    <t>CAP CER 4.7UF 10V X5R 0603</t>
-  </si>
-  <si>
-    <t>CAPC1610X05N</t>
-  </si>
-  <si>
-    <t>490-10477-6-ND</t>
-  </si>
-  <si>
-    <t>GRM1555C1E150JA01D</t>
-  </si>
-  <si>
-    <t>C69, C70</t>
-  </si>
-  <si>
-    <t>15pF</t>
-  </si>
-  <si>
-    <t>CAP CER 15 pF 25V C0G 0402</t>
-  </si>
-  <si>
-    <t>Vishay Lite-On</t>
-  </si>
-  <si>
-    <t>LTST-C155KGJRKT</t>
-  </si>
-  <si>
-    <t>D51, D52, D53</t>
-  </si>
-  <si>
-    <t>LED GREEN/RED CLEAR CHIP SMD</t>
-  </si>
-  <si>
-    <t>160-1409-1-ND</t>
-  </si>
-  <si>
-    <t>ON Semiconductor</t>
-  </si>
-  <si>
-    <t>MBR140SFT1G</t>
-  </si>
-  <si>
-    <t>D50</t>
-  </si>
-  <si>
-    <t>DIODE SCHOTTKY 40V 1A SOD123L</t>
-  </si>
-  <si>
-    <t>SODFL360X110-2N</t>
-  </si>
-  <si>
-    <t>MBR140SFT1GOSDKR-ND</t>
-  </si>
-  <si>
-    <t>NXP Semiconductors</t>
-  </si>
-  <si>
-    <t>PRTR5V0U2F,115</t>
-  </si>
-  <si>
-    <t>U52</t>
-  </si>
-  <si>
-    <t>PRTR5V0U2F</t>
-  </si>
-  <si>
-    <t>TVS DIODE 5.5VWM SOT886</t>
-  </si>
-  <si>
-    <t>SON50P100X50-6N</t>
-  </si>
-  <si>
-    <t>568-4677-6-ND</t>
   </si>
   <si>
     <t>SN74LVC1G17YZPR</t>
@@ -950,7 +950,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{565210E0-A35A-4564-BC25-453C35CDFA05}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2607D05D-3BAC-4B31-A657-B6C2370013C1}">
   <dimension ref="A1:J30"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1228,20 +1228,22 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="C10" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="1">
+        <v>1</v>
+      </c>
+      <c r="E10" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="D10" s="1">
-        <v>3</v>
-      </c>
-      <c r="E10" s="1"/>
       <c r="F10" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>59</v>
@@ -1250,7 +1252,7 @@
         <v>60</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>37</v>
+        <v>19</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>61</v>
@@ -1258,22 +1260,20 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
-        <v>50</v>
+        <v>62</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D11" s="1">
         <v>1</v>
       </c>
-      <c r="E11" s="2" t="s">
-        <v>64</v>
-      </c>
+      <c r="E11" s="1"/>
       <c r="F11" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>65</v>
@@ -1301,287 +1301,285 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="1"/>
+      <c r="E12" s="2" t="s">
+        <v>71</v>
+      </c>
       <c r="F12" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J12" s="2" t="s">
         <v>73</v>
       </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>75</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>76</v>
       </c>
       <c r="D13" s="1">
         <v>2</v>
       </c>
       <c r="E13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>78</v>
-      </c>
       <c r="H13" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="D14" s="1">
         <v>1</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>19</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
+        <v>83</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>85</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="C15" s="2" t="s">
-        <v>87</v>
       </c>
       <c r="D15" s="1">
         <v>4</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>48</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D16" s="1">
         <v>9</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>48</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="D17" s="1">
         <v>1</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H17" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I17" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>100</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B18" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D18" s="1">
+        <v>2</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F18" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="G18" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="H18" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J18" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="D18" s="1">
-        <v>1</v>
-      </c>
-      <c r="E18" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="F18" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>104</v>
-      </c>
-      <c r="H18" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I18" s="1"/>
-      <c r="J18" s="1"/>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="B19" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="D19" s="1">
+        <v>6</v>
+      </c>
+      <c r="E19" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="F19" s="2" t="s">
+        <v>105</v>
+      </c>
+      <c r="G19" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="D19" s="1">
-        <v>2</v>
-      </c>
-      <c r="E19" s="2" t="s">
+      <c r="H19" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J19" s="2" t="s">
         <v>107</v>
-      </c>
-      <c r="F19" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="G19" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="H19" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="I19" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J19" s="2" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
-        <v>74</v>
+        <v>108</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="1">
+        <v>1</v>
+      </c>
+      <c r="E20" s="1"/>
+      <c r="F20" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="G20" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="D20" s="1">
-        <v>6</v>
-      </c>
-      <c r="E20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>112</v>
-      </c>
-      <c r="F20" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G20" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="H20" s="2" t="s">
-        <v>79</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>48</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="C21" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="D21" s="1">
+        <v>14</v>
+      </c>
+      <c r="E21" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="D21" s="1">
-        <v>1</v>
-      </c>
-      <c r="E21" s="1"/>
       <c r="F21" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>118</v>
@@ -1598,221 +1596,219 @@
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="C22" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="D22" s="1">
+        <v>1</v>
+      </c>
+      <c r="E22" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="D22" s="1">
-        <v>14</v>
-      </c>
-      <c r="E22" s="2" t="s">
+      <c r="F22" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="G22" s="2" t="s">
         <v>124</v>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>124</v>
-      </c>
-      <c r="G22" s="2" t="s">
+      <c r="H22" s="2" t="s">
+        <v>119</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="J22" s="2" t="s">
         <v>125</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
-        <v>50</v>
+        <v>114</v>
       </c>
       <c r="B23" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="D23" s="1">
+        <v>6</v>
+      </c>
+      <c r="E23" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="F23" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="G23" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="D23" s="1">
-        <v>1</v>
-      </c>
-      <c r="E23" s="2" t="s">
+      <c r="H23" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>130</v>
-      </c>
-      <c r="G23" s="2" t="s">
+      <c r="I23" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J23" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="H23" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="I23" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="J23" s="2" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
-        <v>121</v>
+        <v>50</v>
       </c>
       <c r="B24" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="D24" s="1">
+        <v>2</v>
+      </c>
+      <c r="E24" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="D24" s="1">
-        <v>6</v>
-      </c>
-      <c r="E24" s="2" t="s">
+      <c r="F24" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="G24" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="G24" s="2" t="s">
-        <v>136</v>
-      </c>
       <c r="H24" s="2" t="s">
-        <v>137</v>
-      </c>
-      <c r="I24" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="J24" s="2" t="s">
-        <v>138</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
-        <v>50</v>
+        <v>136</v>
       </c>
       <c r="B25" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="D25" s="1">
+        <v>3</v>
+      </c>
+      <c r="E25" s="1"/>
+      <c r="F25" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="G25" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="H25" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="J25" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="D25" s="1">
-        <v>2</v>
-      </c>
-      <c r="E25" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="F25" s="2" t="s">
-        <v>141</v>
-      </c>
-      <c r="G25" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="H25" s="2" t="s">
-        <v>126</v>
-      </c>
-      <c r="I25" s="1"/>
-      <c r="J25" s="1"/>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="B26" s="2" t="s">
-        <v>144</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>145</v>
-      </c>
       <c r="D26" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E26" s="1"/>
       <c r="F26" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="G26" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="G26" s="2" t="s">
-        <v>146</v>
-      </c>
       <c r="H26" s="2" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>48</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="C27" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>150</v>
-      </c>
       <c r="D27" s="1">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E27" s="1"/>
       <c r="F27" s="2" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="G27" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="H27" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="H27" s="2" t="s">
+      <c r="I27" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="I27" s="2" t="s">
-        <v>48</v>
-      </c>
       <c r="J27" s="2" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B28" s="2" t="s">
+      <c r="C28" s="2" t="s">
         <v>155</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>156</v>
       </c>
       <c r="D28" s="1">
         <v>1</v>
       </c>
       <c r="E28" s="1"/>
       <c r="F28" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="G28" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="G28" s="2" t="s">
+      <c r="H28" s="2" t="s">
         <v>158</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>159</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>37</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
-        <v>56</v>
+        <v>160</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>161</v>
@@ -1842,7 +1838,7 @@
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
-        <v>56</v>
+        <v>160</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>166</v>

</xml_diff>